<commit_message>
Add __pycache__ to .gitignore
</commit_message>
<xml_diff>
--- a/studio-di-fattibilita/allegati/A1-RTM/RTM-v1.0.xlsx
+++ b/studio-di-fattibilita/allegati/A1-RTM/RTM-v1.0.xlsx
@@ -1043,7 +1043,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>100.0%</t>
         </is>
       </c>
     </row>
@@ -1091,7 +1091,7 @@
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -9884,27 +9884,27 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>StNeed-008</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Comunità Pentema + Garante: no sorveglianza personale, no identificazione volti/targhe in ...</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>ORPHAN ← gap</t>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>SyR-C-003</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>OK (≥1)</t>
         </is>
       </c>
     </row>
@@ -10134,52 +10134,52 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>StNeed-018</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="5" t="inlineStr">
         <is>
           <t>Comune Torriglia: deliberazione formale ospitalità pilota + autorizzazioni locali entro M+...</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>ORPHAN ← gap</t>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>SyR-O-005</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>OK (≥1)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>StNeed-019</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="5" t="inlineStr">
         <is>
           <t>ASL3 Genovese: servizi telemedicina/teleassistenza per residenti Pentema con SLA garantito</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>ORPHAN ← gap</t>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>SyR-F-006</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>OK (≥1)</t>
         </is>
       </c>
     </row>
@@ -10209,52 +10209,52 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>StNeed-021</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="5" t="inlineStr">
         <is>
           <t>MIMIT + ASI + CIRA: posizionamento Firmamento come nodo italiano in roadmap EU HAPS/IRIS²</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>ORPHAN ← gap</t>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>SyR-F-005</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>OK (≥1)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>StNeed-022</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>DTA Puglia + GATB Grottaglie: accesso test bed BVLOS per qualification piattaforma 6A</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>ORPHAN ← gap</t>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>SyR-F-005</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>OK (≥1)</t>
         </is>
       </c>
     </row>
@@ -10384,27 +10384,27 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>StNeed-028</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Firmamento + Coopfond: governance trasparente + audit annuale verso Coopfond + advisory co...</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D29" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="12" t="inlineStr">
-        <is>
-          <t>ORPHAN ← gap</t>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>SyR-Cost-004</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>OK (≥1)</t>
         </is>
       </c>
     </row>
@@ -10450,12 +10450,12 @@
           <t>Orphan StNeeds (no SyR child)</t>
         </is>
       </c>
-      <c r="B2" s="11" t="n">
-        <v>6</v>
+      <c r="B2" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>StNeed-008, StNeed-018, StNeed-019, StNeed-021, StNeed-022, StNeed-028</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -10466,11 +10466,11 @@
         </is>
       </c>
       <c r="B3" s="11" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>SyR-P-002, SyR-P-003, SyR-P-004, SyR-P-005, SyR-P-006, SyR-P-010, SyR-P-011, SyR-P-012, SyR-O-002, SyR-O-006, SyR-O-008, SyR-S-003, SyR-S-005, SyR-C-005, SyR-C-006, SyR-C-009, SyR-C-010, SyR-C-012, SyR-Cost-005, SyR-Cost-007, SyR-Cost-008, SyR-Cost-009</t>
+          <t>SyR-C-005</t>
         </is>
       </c>
     </row>
@@ -10527,7 +10527,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>78.6%</t>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -13280,12 +13280,12 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Boundary B2 + visione strategica 6B</t>
+          <t>Boundary B2 + visione strategica 6B + nodo italiano EU HAPS StNeed-021 + test bed GATB StNeed-022</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>StNeed-017,StNeed-023</t>
+          <t>StNeed-017,StNeed-021,StNeed-022,StNeed-023</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -13295,7 +13295,7 @@
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
-          <t>StNeed-017,StNeed-023</t>
+          <t>StNeed-017,StNeed-021,StNeed-022,StNeed-023</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -13352,17 +13352,17 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>Sistema [6A] supporta SAR persone disperse con osservazione aerea persistente &gt;2h + payload IR</t>
+          <t>Sistema [6A] supporta SAR persone disperse con osservazione aerea persistente &gt;2h + payload IR + telemedicina rurale link UC-008</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Supporto StNeed-004</t>
+          <t>Supporto StNeed-004 + StNeed-019 ASL3 telemedicina</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>StNeed-004</t>
+          <t>StNeed-004,StNeed-019</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -13372,7 +13372,7 @@
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>StNeed-004</t>
+          <t>StNeed-004,StNeed-019</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
@@ -14974,12 +14974,12 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Compliance ENAC + sicurezza StNeed-011 + HR StNeed-026</t>
+          <t>Compliance ENAC + sicurezza + HR StNeed-026 + Comune Torriglia StNeed-018</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
         <is>
-          <t>StNeed-011,StNeed-026 + Reg.APR Ed.3</t>
+          <t>StNeed-011,StNeed-026,StNeed-018 + Reg.APR Ed.3</t>
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr">
@@ -14989,7 +14989,7 @@
       </c>
       <c r="F28" s="9" t="inlineStr">
         <is>
-          <t>StNeed-011,StNeed-026</t>
+          <t>StNeed-011,StNeed-026,StNeed-018</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
@@ -16437,12 +16437,12 @@
       </c>
       <c r="C47" s="9" t="inlineStr">
         <is>
-          <t>StNeed-014 + Cap.5.6</t>
+          <t>StNeed-014 + StNeed-008 + Cap.5.6</t>
         </is>
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>StNeed-014</t>
+          <t>StNeed-014,StNeed-008</t>
         </is>
       </c>
       <c r="E47" s="9" t="inlineStr">
@@ -16452,7 +16452,7 @@
       </c>
       <c r="F47" s="9" t="inlineStr">
         <is>
-          <t>StNeed-014</t>
+          <t>StNeed-014,StNeed-008</t>
         </is>
       </c>
       <c r="G47" s="9" t="inlineStr">
@@ -17433,17 +17433,17 @@
       </c>
       <c r="B60" s="9" t="inlineStr">
         <is>
-          <t>Modello servizio ricorrente (DaaS/IaaS/canone) — no vendita asset</t>
+          <t>Modello servizio ricorrente (DaaS/IaaS/canone) — no vendita asset + governance trasparente verso Coopfond</t>
         </is>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>StNeed-015 + boundary B1</t>
+          <t>StNeed-015 + StNeed-028 governance + boundary B1</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>StNeed-015 + B1</t>
+          <t>StNeed-015,StNeed-028 + B1</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
@@ -17453,7 +17453,7 @@
       </c>
       <c r="F60" s="9" t="inlineStr">
         <is>
-          <t>StNeed-015</t>
+          <t>StNeed-015,StNeed-028</t>
         </is>
       </c>
       <c r="G60" s="9" t="inlineStr">

</xml_diff>